<commit_message>
docs: actualizar Gantt S23 + agregar fuentes Excel de costos
Gantt Semana 23:
- S2 marcado ✓ Jue 05 en hoja Semana 23
- Plan Santiago: S2 en PRIORIDAD 2 marcado ✓, notas ampliadas
  con descripción completa del trabajo (costos + desglose collapsible)
- S2 agregado al bloque COMPLETADOS con descripción técnica
- S2 eliminado de PRÓXIMO (ya completado)

Archivos fuente nuevos:
- Bases de datos/DASHBOARD COSTOS ABRIL.xlsx — dashboard Excel de
  referencia para B2 (hoja GRAFICAS con 4 charts + tablas estadísticas)
- Bases de datos/cajitas.xlsx — fuente de costos COP/m³ por fase
  (CONS POR FASE, CONS POR LINEA, EQUIPOS) usada en S2

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gantt/Gantt Semana 23 - App PTAR.xlsx
+++ b/Gantt/Gantt Semana 23 - App PTAR.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Semana 23" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Plan Santiago" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semana 23" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan Santiago" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -419,7 +419,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -576,6 +576,15 @@
     <xf numFmtId="0" fontId="25" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1051,7 +1060,7 @@
       <c r="G5" s="13" t="n"/>
     </row>
     <row r="6" ht="24" customHeight="1" s="34">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="60" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
@@ -1066,18 +1075,14 @@
           <t>Santiago</t>
         </is>
       </c>
-      <c r="D6" s="17" t="inlineStr">
-        <is>
-          <t>▶</t>
-        </is>
-      </c>
-      <c r="E6" s="17" t="inlineStr">
-        <is>
-          <t>◀</t>
-        </is>
-      </c>
+      <c r="D6" s="66" t="n"/>
+      <c r="E6" s="66" t="n"/>
       <c r="F6" s="18" t="n"/>
-      <c r="G6" s="19" t="n"/>
+      <c r="G6" s="67" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="24" customHeight="1" s="34">
       <c r="A7" s="8" t="inlineStr">
@@ -1901,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="34" min="1" max="1"/>
@@ -2274,7 +2279,7 @@
       <c r="F13" s="47" t="n"/>
     </row>
     <row r="14" ht="42" customHeight="1" s="34">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="48" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
@@ -2298,14 +2303,20 @@
           <t>Splash / Diagrama</t>
         </is>
       </c>
-      <c r="E14" s="30" t="inlineStr">
-        <is>
-          <t>Lun–Mar</t>
+      <c r="E14" s="68" t="inlineStr">
+        <is>
+          <t>Jue 05 ✓</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>CONS POR FASE: PRELIM $1.138/m³ · PRIMARIA $6.757 · SECUNDARIA $3.204 · TERCIARIA $2.807. También disponible por línea (CONS POR LINEA). Zoom ya está implementado, no tocar.</t>
+          <t>COMPLETADO. Dos fases:
+1. Costos reales COP/m³ desde cajitas.xlsx (CONS POR LINEA + CONS POR FASE):
+   PRELIM .138 · PRIM .757 · SEC .204 · TERC .807
+2. Desglose collapsible en modal equipo (doble-clic):
+   • COSTOS DEL EQUIPO: energía exacta kW, lavTK, químicos (19 equipos)
+   • COSTOS COMPARTIDOS: nómina 85, membranas, residuos por fase
+Commits: 8890a30 (costos) + 1febb97 (desglose)</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2751,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="51" t="inlineStr">
         <is>
@@ -2879,8 +2889,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="56" t="inlineStr">
         <is>
@@ -3016,7 +3024,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="63" t="inlineStr">
         <is>
@@ -3160,58 +3167,44 @@
         </is>
       </c>
     </row>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57">
-      <c r="A57" s="56" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="52" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B55" s="64" t="inlineStr">
+        <is>
+          <t>Costos reales COP/m³ (cajitas.xlsx) + desglose collapsible por equipo y fase en modal — CONS POR LINEA: energía kW, lavTK, químicos · CONS POR FASE: nómina, membranas, residuos</t>
+        </is>
+      </c>
+      <c r="E55" s="55" t="inlineStr">
+        <is>
+          <t>Jue 05 ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="56" t="inlineStr">
         <is>
           <t>🔜  PRÓXIMO — Prioridad 2</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="57" t="inlineStr">
-        <is>
-          <t>S2</t>
-        </is>
-      </c>
-      <c r="B58" s="58" t="inlineStr">
-        <is>
-          <t>Actualizar costos splash por fase/equipo ($COP/m³ reales desde cajitas.xlsx)</t>
-        </is>
-      </c>
-      <c r="E58" s="65" t="inlineStr">
-        <is>
-          <t>Post S23</t>
-        </is>
-      </c>
-    </row>
     <row r="59">
-      <c r="A59" s="57" t="inlineStr">
-        <is>
-          <t>R3</t>
-        </is>
-      </c>
-      <c r="B59" s="58" t="inlineStr">
-        <is>
-          <t>Implementar campos nuevos formulario RO (depende R1 de Luna)</t>
-        </is>
-      </c>
-      <c r="E59" s="65" t="inlineStr">
-        <is>
-          <t>Post S23</t>
-        </is>
-      </c>
+      <c r="A59" s="55" t="n"/>
+      <c r="B59" s="58" t="n"/>
+      <c r="E59" s="55" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="57" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B60" s="58" t="inlineStr">
         <is>
-          <t>Agregar $/m³ por reactivo RO (depende R3)</t>
+          <t>Implementar campos nuevos formulario RO (depende R1 de Luna)</t>
         </is>
       </c>
       <c r="E60" s="65" t="inlineStr">
@@ -3223,12 +3216,12 @@
     <row r="61">
       <c r="A61" s="57" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B61" s="58" t="inlineStr">
         <is>
-          <t>Conexión balance químico BD + gráficas CostosDashboard</t>
+          <t>Agregar $/m³ por reactivo RO (depende R3)</t>
         </is>
       </c>
       <c r="E61" s="65" t="inlineStr">
@@ -3240,15 +3233,32 @@
     <row r="62">
       <c r="A62" s="57" t="inlineStr">
         <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B62" s="58" t="inlineStr">
+        <is>
+          <t>Conexión balance químico BD + gráficas CostosDashboard</t>
+        </is>
+      </c>
+      <c r="E62" s="65" t="inlineStr">
+        <is>
+          <t>Post S23</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="57" t="inlineStr">
+        <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B62" s="58" t="inlineStr">
+      <c r="B63" s="58" t="inlineStr">
         <is>
           <t>Tablas resumen bajo gráficas de costos</t>
         </is>
       </c>
-      <c r="E62" s="65" t="inlineStr">
+      <c r="E63" s="65" t="inlineStr">
         <is>
           <t>Post S23</t>
         </is>

</xml_diff>